<commit_message>
Deep dive, layout, logo, motion and Genie refinements
- KPI deep dive: fixed dialog size across tabs, Plan buttons to open any
  state or channel plan, sharpest growth banner removed, one to two line
  insight closing every tab; growth metrics are never flagged red
- Remove hot and hotspot wording from the UI and workbook
- Full width content, sidebar toggle in the top bar, More panel holding
  the Sales to Install Journey
- Brightspeed logo mark and wordmark
- Smoother compositor only motion: page and dialog transitions, eased
  hover lifts; removed repaint heavy effects
- Insights Genie: short thinking pause with a spinning mark and status
  messages

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/Brightspeed_Cancellation_Data_Jan_Sep_2026.xlsx
+++ b/data/Brightspeed_Cancellation_Data_Jan_Sep_2026.xlsx
@@ -203,7 +203,7 @@
     <t>Cancelled while Tech on Job</t>
   </si>
   <si>
-    <t>North Carolina: September hotspot</t>
+    <t>North Carolina: September focus state</t>
   </si>
   <si>
     <t>Metric</t>
@@ -356,7 +356,7 @@
     <t>September 2026 State Comparison</t>
   </si>
   <si>
-    <t>North Carolina is the primary hotspot; all other states remain within their normal range.</t>
+    <t>North Carolina is the primary focus state; all other states remain within their normal range.</t>
   </si>
   <si>
     <t>Cancellation Timing: Pre ODD, On ODD, Post ODD</t>
@@ -404,7 +404,7 @@
     <t>Elevated</t>
   </si>
   <si>
-    <t>September hotspot</t>
+    <t>September focus</t>
   </si>
   <si>
     <t>Customers unavailable at the appointment; confirm access the day before.</t>
@@ -431,7 +431,7 @@
     <t>Consistent with normal operating range</t>
   </si>
   <si>
-    <t>Primary customer contact hotspot</t>
+    <t>Primary customer contact concentration</t>
   </si>
   <si>
     <t>Portfolio</t>

</xml_diff>